<commit_message>
Designazioni API: READY status e endpoint send-person/send-period
</commit_message>
<xml_diff>
--- a/data/DB_PITCH_2.xlsx
+++ b/data/DB_PITCH_2.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dazngroup-my.sharepoint.com/personal/andrea_andrisano_dazn_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="351" documentId="8_{E638DADE-4357-7740-8B3F-AF5E8C45027C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FB122A7-1B6D-584C-AC70-2E4DCDE5ADEB}"/>
+  <xr:revisionPtr revIDLastSave="580" documentId="8_{E638DADE-4357-7740-8B3F-AF5E8C45027C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2239CA35-23B6-4349-BB81-439FD4A787CC}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ROLES" sheetId="3" r:id="rId1"/>
     <sheet name="STAFF" sheetId="2" r:id="rId2"/>
     <sheet name="EVENTS" sheetId="4" r:id="rId3"/>
+    <sheet name="STANDARD_REQUIREMENTS" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="267">
   <si>
     <t>RIZZO</t>
   </si>
@@ -724,6 +725,105 @@
   </si>
   <si>
     <t>competition_name</t>
+  </si>
+  <si>
+    <t>PCR02</t>
+  </si>
+  <si>
+    <t>PCR03</t>
+  </si>
+  <si>
+    <t>DAZN1</t>
+  </si>
+  <si>
+    <t>GALLERY02</t>
+  </si>
+  <si>
+    <t>GALLERY03</t>
+  </si>
+  <si>
+    <t>DAZN2</t>
+  </si>
+  <si>
+    <t>site</t>
+  </si>
+  <si>
+    <t>role_code</t>
+  </si>
+  <si>
+    <t>PCR</t>
+  </si>
+  <si>
+    <t>GALLERY</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>GALLERY04</t>
+  </si>
+  <si>
+    <t>NO STADIO</t>
+  </si>
+  <si>
+    <t>BOOTH1</t>
+  </si>
+  <si>
+    <t>BOOTH2</t>
+  </si>
+  <si>
+    <t>BOOTH3</t>
+  </si>
+  <si>
+    <t>BOOTH4</t>
+  </si>
+  <si>
+    <t>BOOTH5</t>
+  </si>
+  <si>
+    <t>BOOTH6</t>
+  </si>
+  <si>
+    <t>BOOTH7</t>
+  </si>
+  <si>
+    <t>BOOTH8</t>
+  </si>
+  <si>
+    <t>BOOTH9</t>
+  </si>
+  <si>
+    <t>BOOTH10</t>
+  </si>
+  <si>
+    <t>BOOTH11</t>
+  </si>
+  <si>
+    <t>BOOTH12</t>
+  </si>
+  <si>
+    <t>WORLD FEED</t>
+  </si>
+  <si>
+    <t>VODCAST</t>
+  </si>
+  <si>
+    <t>REALIZZATORE VMIX</t>
+  </si>
+  <si>
+    <t>BLU STUDIO</t>
+  </si>
+  <si>
+    <t>SIMPLY</t>
+  </si>
+  <si>
+    <t>VMIX1</t>
+  </si>
+  <si>
+    <t>Simply</t>
+  </si>
+  <si>
+    <t>Realizzatore Vmix</t>
   </si>
 </sst>
 </file>
@@ -733,7 +833,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -758,6 +858,20 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -811,7 +925,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -841,6 +955,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1145,7 +1260,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.5" style="2" customWidth="1"/>
@@ -1842,6 +1957,34 @@
       </c>
       <c r="D49" s="3" t="s">
         <v>87</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="2">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="2">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -2780,6 +2923,4327 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F145EDD5-84E4-D742-B889-26407727CF3D}">
+  <dimension ref="A1:G215"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="5" width="30.5" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" style="3" customWidth="1"/>
+    <col min="7" max="8" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>236</v>
+      </c>
+      <c r="B3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" t="s">
+        <v>242</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" t="s">
+        <v>242</v>
+      </c>
+      <c r="D6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>236</v>
+      </c>
+      <c r="B8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" t="s">
+        <v>242</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>236</v>
+      </c>
+      <c r="B9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C9" t="s">
+        <v>242</v>
+      </c>
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>236</v>
+      </c>
+      <c r="B10" t="s">
+        <v>234</v>
+      </c>
+      <c r="C10" t="s">
+        <v>242</v>
+      </c>
+      <c r="D10" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" t="s">
+        <v>87</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>236</v>
+      </c>
+      <c r="B11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C11" t="s">
+        <v>242</v>
+      </c>
+      <c r="D11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>236</v>
+      </c>
+      <c r="B12" t="s">
+        <v>234</v>
+      </c>
+      <c r="C12" t="s">
+        <v>242</v>
+      </c>
+      <c r="D12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" t="s">
+        <v>87</v>
+      </c>
+      <c r="F12" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>236</v>
+      </c>
+      <c r="B13" t="s">
+        <v>234</v>
+      </c>
+      <c r="C13" t="s">
+        <v>242</v>
+      </c>
+      <c r="D13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>236</v>
+      </c>
+      <c r="B14" t="s">
+        <v>234</v>
+      </c>
+      <c r="C14" t="s">
+        <v>242</v>
+      </c>
+      <c r="D14" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14" t="s">
+        <v>87</v>
+      </c>
+      <c r="F14" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>236</v>
+      </c>
+      <c r="B15" t="s">
+        <v>234</v>
+      </c>
+      <c r="C15" t="s">
+        <v>242</v>
+      </c>
+      <c r="D15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>236</v>
+      </c>
+      <c r="B16" t="s">
+        <v>234</v>
+      </c>
+      <c r="C16" t="s">
+        <v>242</v>
+      </c>
+      <c r="D16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>236</v>
+      </c>
+      <c r="B17" t="s">
+        <v>234</v>
+      </c>
+      <c r="C17" t="s">
+        <v>242</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>236</v>
+      </c>
+      <c r="B18" t="s">
+        <v>235</v>
+      </c>
+      <c r="C18" t="s">
+        <v>242</v>
+      </c>
+      <c r="D18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" t="s">
+        <v>87</v>
+      </c>
+      <c r="F18" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>236</v>
+      </c>
+      <c r="B19" t="s">
+        <v>235</v>
+      </c>
+      <c r="C19" t="s">
+        <v>242</v>
+      </c>
+      <c r="D19" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>236</v>
+      </c>
+      <c r="B20" t="s">
+        <v>235</v>
+      </c>
+      <c r="C20" t="s">
+        <v>242</v>
+      </c>
+      <c r="D20" t="s">
+        <v>89</v>
+      </c>
+      <c r="E20" t="s">
+        <v>87</v>
+      </c>
+      <c r="F20" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>236</v>
+      </c>
+      <c r="B21" t="s">
+        <v>235</v>
+      </c>
+      <c r="C21" t="s">
+        <v>242</v>
+      </c>
+      <c r="D21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>236</v>
+      </c>
+      <c r="B22" t="s">
+        <v>235</v>
+      </c>
+      <c r="C22" t="s">
+        <v>242</v>
+      </c>
+      <c r="D22" t="s">
+        <v>97</v>
+      </c>
+      <c r="E22" t="s">
+        <v>87</v>
+      </c>
+      <c r="F22" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>236</v>
+      </c>
+      <c r="B23" t="s">
+        <v>235</v>
+      </c>
+      <c r="C23" t="s">
+        <v>242</v>
+      </c>
+      <c r="D23" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>236</v>
+      </c>
+      <c r="B24" t="s">
+        <v>235</v>
+      </c>
+      <c r="C24" t="s">
+        <v>242</v>
+      </c>
+      <c r="D24" t="s">
+        <v>50</v>
+      </c>
+      <c r="E24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>236</v>
+      </c>
+      <c r="B25" t="s">
+        <v>235</v>
+      </c>
+      <c r="C25" t="s">
+        <v>242</v>
+      </c>
+      <c r="D25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>236</v>
+      </c>
+      <c r="B26" t="s">
+        <v>113</v>
+      </c>
+      <c r="C26" t="s">
+        <v>243</v>
+      </c>
+      <c r="D26" t="s">
+        <v>98</v>
+      </c>
+      <c r="E26" t="s">
+        <v>87</v>
+      </c>
+      <c r="F26" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>236</v>
+      </c>
+      <c r="B27" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" t="s">
+        <v>243</v>
+      </c>
+      <c r="D27" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>236</v>
+      </c>
+      <c r="B28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" t="s">
+        <v>243</v>
+      </c>
+      <c r="D28" t="s">
+        <v>88</v>
+      </c>
+      <c r="E28" t="s">
+        <v>87</v>
+      </c>
+      <c r="F28" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>236</v>
+      </c>
+      <c r="B29" t="s">
+        <v>113</v>
+      </c>
+      <c r="C29" t="s">
+        <v>243</v>
+      </c>
+      <c r="D29" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>236</v>
+      </c>
+      <c r="B30" t="s">
+        <v>113</v>
+      </c>
+      <c r="C30" t="s">
+        <v>243</v>
+      </c>
+      <c r="D30" t="s">
+        <v>80</v>
+      </c>
+      <c r="E30" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>236</v>
+      </c>
+      <c r="B31" t="s">
+        <v>113</v>
+      </c>
+      <c r="C31" t="s">
+        <v>243</v>
+      </c>
+      <c r="D31" t="s">
+        <v>79</v>
+      </c>
+      <c r="E31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F31" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>236</v>
+      </c>
+      <c r="B32" t="s">
+        <v>113</v>
+      </c>
+      <c r="C32" t="s">
+        <v>243</v>
+      </c>
+      <c r="D32" t="s">
+        <v>81</v>
+      </c>
+      <c r="E32" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>236</v>
+      </c>
+      <c r="B33" t="s">
+        <v>113</v>
+      </c>
+      <c r="C33" t="s">
+        <v>243</v>
+      </c>
+      <c r="D33" t="s">
+        <v>89</v>
+      </c>
+      <c r="E33" t="s">
+        <v>87</v>
+      </c>
+      <c r="F33" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>236</v>
+      </c>
+      <c r="B34" t="s">
+        <v>113</v>
+      </c>
+      <c r="C34" t="s">
+        <v>243</v>
+      </c>
+      <c r="D34" t="s">
+        <v>22</v>
+      </c>
+      <c r="E34" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>236</v>
+      </c>
+      <c r="B35" t="s">
+        <v>113</v>
+      </c>
+      <c r="C35" t="s">
+        <v>243</v>
+      </c>
+      <c r="D35" t="s">
+        <v>97</v>
+      </c>
+      <c r="E35" t="s">
+        <v>87</v>
+      </c>
+      <c r="F35" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>236</v>
+      </c>
+      <c r="B36" t="s">
+        <v>113</v>
+      </c>
+      <c r="C36" t="s">
+        <v>243</v>
+      </c>
+      <c r="D36" t="s">
+        <v>29</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>236</v>
+      </c>
+      <c r="B37" t="s">
+        <v>113</v>
+      </c>
+      <c r="C37" t="s">
+        <v>243</v>
+      </c>
+      <c r="D37" t="s">
+        <v>15</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>236</v>
+      </c>
+      <c r="B38" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" t="s">
+        <v>243</v>
+      </c>
+      <c r="D38" t="s">
+        <v>50</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>236</v>
+      </c>
+      <c r="B39" t="s">
+        <v>113</v>
+      </c>
+      <c r="C39" t="s">
+        <v>243</v>
+      </c>
+      <c r="D39" t="s">
+        <v>7</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>236</v>
+      </c>
+      <c r="B40" t="s">
+        <v>237</v>
+      </c>
+      <c r="C40" t="s">
+        <v>243</v>
+      </c>
+      <c r="D40" t="s">
+        <v>98</v>
+      </c>
+      <c r="E40" t="s">
+        <v>87</v>
+      </c>
+      <c r="F40" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>236</v>
+      </c>
+      <c r="B41" t="s">
+        <v>237</v>
+      </c>
+      <c r="C41" t="s">
+        <v>243</v>
+      </c>
+      <c r="D41" t="s">
+        <v>75</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>236</v>
+      </c>
+      <c r="B42" t="s">
+        <v>237</v>
+      </c>
+      <c r="C42" t="s">
+        <v>243</v>
+      </c>
+      <c r="D42" t="s">
+        <v>88</v>
+      </c>
+      <c r="E42" t="s">
+        <v>87</v>
+      </c>
+      <c r="F42" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>236</v>
+      </c>
+      <c r="B43" t="s">
+        <v>237</v>
+      </c>
+      <c r="C43" t="s">
+        <v>243</v>
+      </c>
+      <c r="D43" t="s">
+        <v>57</v>
+      </c>
+      <c r="E43" t="s">
+        <v>8</v>
+      </c>
+      <c r="F43" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>236</v>
+      </c>
+      <c r="B44" t="s">
+        <v>237</v>
+      </c>
+      <c r="C44" t="s">
+        <v>243</v>
+      </c>
+      <c r="D44" t="s">
+        <v>80</v>
+      </c>
+      <c r="E44" t="s">
+        <v>8</v>
+      </c>
+      <c r="F44" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>236</v>
+      </c>
+      <c r="B45" t="s">
+        <v>237</v>
+      </c>
+      <c r="C45" t="s">
+        <v>243</v>
+      </c>
+      <c r="D45" t="s">
+        <v>79</v>
+      </c>
+      <c r="E45" t="s">
+        <v>8</v>
+      </c>
+      <c r="F45" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>236</v>
+      </c>
+      <c r="B46" t="s">
+        <v>237</v>
+      </c>
+      <c r="C46" t="s">
+        <v>243</v>
+      </c>
+      <c r="D46" t="s">
+        <v>81</v>
+      </c>
+      <c r="E46" t="s">
+        <v>8</v>
+      </c>
+      <c r="F46" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>236</v>
+      </c>
+      <c r="B47" t="s">
+        <v>237</v>
+      </c>
+      <c r="C47" t="s">
+        <v>243</v>
+      </c>
+      <c r="D47" t="s">
+        <v>89</v>
+      </c>
+      <c r="E47" t="s">
+        <v>87</v>
+      </c>
+      <c r="F47" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>236</v>
+      </c>
+      <c r="B48" t="s">
+        <v>237</v>
+      </c>
+      <c r="C48" t="s">
+        <v>243</v>
+      </c>
+      <c r="D48" t="s">
+        <v>22</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>236</v>
+      </c>
+      <c r="B49" t="s">
+        <v>237</v>
+      </c>
+      <c r="C49" t="s">
+        <v>243</v>
+      </c>
+      <c r="D49" t="s">
+        <v>97</v>
+      </c>
+      <c r="E49" t="s">
+        <v>87</v>
+      </c>
+      <c r="F49" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>236</v>
+      </c>
+      <c r="B50" t="s">
+        <v>237</v>
+      </c>
+      <c r="C50" t="s">
+        <v>243</v>
+      </c>
+      <c r="D50" t="s">
+        <v>29</v>
+      </c>
+      <c r="E50" t="s">
+        <v>8</v>
+      </c>
+      <c r="F50" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>236</v>
+      </c>
+      <c r="B51" t="s">
+        <v>237</v>
+      </c>
+      <c r="C51" t="s">
+        <v>243</v>
+      </c>
+      <c r="D51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E51" t="s">
+        <v>8</v>
+      </c>
+      <c r="F51" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>236</v>
+      </c>
+      <c r="B52" t="s">
+        <v>237</v>
+      </c>
+      <c r="C52" t="s">
+        <v>243</v>
+      </c>
+      <c r="D52" t="s">
+        <v>50</v>
+      </c>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+      <c r="F52" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>236</v>
+      </c>
+      <c r="B53" t="s">
+        <v>237</v>
+      </c>
+      <c r="C53" t="s">
+        <v>243</v>
+      </c>
+      <c r="D53" t="s">
+        <v>7</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>236</v>
+      </c>
+      <c r="B54" t="s">
+        <v>238</v>
+      </c>
+      <c r="C54" t="s">
+        <v>243</v>
+      </c>
+      <c r="D54" t="s">
+        <v>98</v>
+      </c>
+      <c r="E54" t="s">
+        <v>87</v>
+      </c>
+      <c r="F54" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>236</v>
+      </c>
+      <c r="B55" t="s">
+        <v>238</v>
+      </c>
+      <c r="C55" t="s">
+        <v>243</v>
+      </c>
+      <c r="D55" t="s">
+        <v>75</v>
+      </c>
+      <c r="E55" t="s">
+        <v>8</v>
+      </c>
+      <c r="F55" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>236</v>
+      </c>
+      <c r="B56" t="s">
+        <v>238</v>
+      </c>
+      <c r="C56" t="s">
+        <v>243</v>
+      </c>
+      <c r="D56" t="s">
+        <v>88</v>
+      </c>
+      <c r="E56" t="s">
+        <v>87</v>
+      </c>
+      <c r="F56" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>236</v>
+      </c>
+      <c r="B57" t="s">
+        <v>238</v>
+      </c>
+      <c r="C57" t="s">
+        <v>243</v>
+      </c>
+      <c r="D57" t="s">
+        <v>57</v>
+      </c>
+      <c r="E57" t="s">
+        <v>8</v>
+      </c>
+      <c r="F57" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>236</v>
+      </c>
+      <c r="B58" t="s">
+        <v>238</v>
+      </c>
+      <c r="C58" t="s">
+        <v>243</v>
+      </c>
+      <c r="D58" t="s">
+        <v>263</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>236</v>
+      </c>
+      <c r="B59" t="s">
+        <v>238</v>
+      </c>
+      <c r="C59" t="s">
+        <v>243</v>
+      </c>
+      <c r="D59" t="s">
+        <v>79</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>236</v>
+      </c>
+      <c r="B60" t="s">
+        <v>238</v>
+      </c>
+      <c r="C60" t="s">
+        <v>243</v>
+      </c>
+      <c r="D60" t="s">
+        <v>81</v>
+      </c>
+      <c r="E60" t="s">
+        <v>8</v>
+      </c>
+      <c r="F60" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>236</v>
+      </c>
+      <c r="B61" t="s">
+        <v>238</v>
+      </c>
+      <c r="C61" t="s">
+        <v>243</v>
+      </c>
+      <c r="D61" t="s">
+        <v>89</v>
+      </c>
+      <c r="E61" t="s">
+        <v>87</v>
+      </c>
+      <c r="F61" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>236</v>
+      </c>
+      <c r="B62" t="s">
+        <v>238</v>
+      </c>
+      <c r="C62" t="s">
+        <v>243</v>
+      </c>
+      <c r="D62" t="s">
+        <v>22</v>
+      </c>
+      <c r="E62" t="s">
+        <v>8</v>
+      </c>
+      <c r="F62" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>236</v>
+      </c>
+      <c r="B63" t="s">
+        <v>238</v>
+      </c>
+      <c r="C63" t="s">
+        <v>243</v>
+      </c>
+      <c r="D63" t="s">
+        <v>97</v>
+      </c>
+      <c r="E63" t="s">
+        <v>87</v>
+      </c>
+      <c r="F63" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>236</v>
+      </c>
+      <c r="B64" t="s">
+        <v>238</v>
+      </c>
+      <c r="C64" t="s">
+        <v>243</v>
+      </c>
+      <c r="D64" t="s">
+        <v>29</v>
+      </c>
+      <c r="E64" t="s">
+        <v>8</v>
+      </c>
+      <c r="F64" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>236</v>
+      </c>
+      <c r="B65" t="s">
+        <v>238</v>
+      </c>
+      <c r="C65" t="s">
+        <v>243</v>
+      </c>
+      <c r="D65" t="s">
+        <v>15</v>
+      </c>
+      <c r="E65" t="s">
+        <v>8</v>
+      </c>
+      <c r="F65" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>236</v>
+      </c>
+      <c r="B66" t="s">
+        <v>238</v>
+      </c>
+      <c r="C66" t="s">
+        <v>243</v>
+      </c>
+      <c r="D66" t="s">
+        <v>50</v>
+      </c>
+      <c r="E66" t="s">
+        <v>8</v>
+      </c>
+      <c r="F66" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>236</v>
+      </c>
+      <c r="B67" t="s">
+        <v>238</v>
+      </c>
+      <c r="C67" t="s">
+        <v>243</v>
+      </c>
+      <c r="D67" t="s">
+        <v>7</v>
+      </c>
+      <c r="E67" t="s">
+        <v>8</v>
+      </c>
+      <c r="F67" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>239</v>
+      </c>
+      <c r="B68" t="s">
+        <v>113</v>
+      </c>
+      <c r="C68" t="s">
+        <v>243</v>
+      </c>
+      <c r="D68" t="s">
+        <v>73</v>
+      </c>
+      <c r="E68" t="s">
+        <v>87</v>
+      </c>
+      <c r="F68" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>239</v>
+      </c>
+      <c r="B69" t="s">
+        <v>113</v>
+      </c>
+      <c r="C69" t="s">
+        <v>243</v>
+      </c>
+      <c r="D69" t="s">
+        <v>75</v>
+      </c>
+      <c r="E69" t="s">
+        <v>8</v>
+      </c>
+      <c r="F69" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>239</v>
+      </c>
+      <c r="B70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C70" t="s">
+        <v>243</v>
+      </c>
+      <c r="D70" t="s">
+        <v>88</v>
+      </c>
+      <c r="E70" t="s">
+        <v>87</v>
+      </c>
+      <c r="F70" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>239</v>
+      </c>
+      <c r="B71" t="s">
+        <v>113</v>
+      </c>
+      <c r="C71" t="s">
+        <v>243</v>
+      </c>
+      <c r="D71" t="s">
+        <v>57</v>
+      </c>
+      <c r="E71" t="s">
+        <v>8</v>
+      </c>
+      <c r="F71" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>239</v>
+      </c>
+      <c r="B72" t="s">
+        <v>113</v>
+      </c>
+      <c r="C72" t="s">
+        <v>243</v>
+      </c>
+      <c r="D72" t="s">
+        <v>80</v>
+      </c>
+      <c r="E72" t="s">
+        <v>8</v>
+      </c>
+      <c r="F72" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>239</v>
+      </c>
+      <c r="B73" t="s">
+        <v>113</v>
+      </c>
+      <c r="C73" t="s">
+        <v>243</v>
+      </c>
+      <c r="D73" t="s">
+        <v>79</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>239</v>
+      </c>
+      <c r="B74" t="s">
+        <v>113</v>
+      </c>
+      <c r="C74" t="s">
+        <v>243</v>
+      </c>
+      <c r="D74" t="s">
+        <v>81</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>239</v>
+      </c>
+      <c r="B75" t="s">
+        <v>113</v>
+      </c>
+      <c r="C75" t="s">
+        <v>243</v>
+      </c>
+      <c r="D75" t="s">
+        <v>89</v>
+      </c>
+      <c r="E75" t="s">
+        <v>87</v>
+      </c>
+      <c r="F75" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>239</v>
+      </c>
+      <c r="B76" t="s">
+        <v>113</v>
+      </c>
+      <c r="C76" t="s">
+        <v>243</v>
+      </c>
+      <c r="D76" t="s">
+        <v>22</v>
+      </c>
+      <c r="E76" t="s">
+        <v>8</v>
+      </c>
+      <c r="F76" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>239</v>
+      </c>
+      <c r="B77" t="s">
+        <v>113</v>
+      </c>
+      <c r="C77" t="s">
+        <v>243</v>
+      </c>
+      <c r="D77" t="s">
+        <v>29</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>239</v>
+      </c>
+      <c r="B78" t="s">
+        <v>113</v>
+      </c>
+      <c r="C78" t="s">
+        <v>243</v>
+      </c>
+      <c r="D78" t="s">
+        <v>15</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>239</v>
+      </c>
+      <c r="B79" t="s">
+        <v>113</v>
+      </c>
+      <c r="C79" t="s">
+        <v>243</v>
+      </c>
+      <c r="D79" t="s">
+        <v>50</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>239</v>
+      </c>
+      <c r="B80" t="s">
+        <v>113</v>
+      </c>
+      <c r="C80" t="s">
+        <v>243</v>
+      </c>
+      <c r="D80" t="s">
+        <v>90</v>
+      </c>
+      <c r="E80" t="s">
+        <v>87</v>
+      </c>
+      <c r="F80" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>239</v>
+      </c>
+      <c r="B81" t="s">
+        <v>113</v>
+      </c>
+      <c r="C81" t="s">
+        <v>243</v>
+      </c>
+      <c r="D81" t="s">
+        <v>7</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>239</v>
+      </c>
+      <c r="B82" t="s">
+        <v>237</v>
+      </c>
+      <c r="C82" t="s">
+        <v>243</v>
+      </c>
+      <c r="D82" t="s">
+        <v>73</v>
+      </c>
+      <c r="E82" t="s">
+        <v>87</v>
+      </c>
+      <c r="F82" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>239</v>
+      </c>
+      <c r="B83" t="s">
+        <v>237</v>
+      </c>
+      <c r="C83" t="s">
+        <v>243</v>
+      </c>
+      <c r="D83" t="s">
+        <v>75</v>
+      </c>
+      <c r="E83" t="s">
+        <v>8</v>
+      </c>
+      <c r="F83" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>239</v>
+      </c>
+      <c r="B84" t="s">
+        <v>237</v>
+      </c>
+      <c r="C84" t="s">
+        <v>243</v>
+      </c>
+      <c r="D84" t="s">
+        <v>88</v>
+      </c>
+      <c r="E84" t="s">
+        <v>87</v>
+      </c>
+      <c r="F84" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>239</v>
+      </c>
+      <c r="B85" t="s">
+        <v>237</v>
+      </c>
+      <c r="C85" t="s">
+        <v>243</v>
+      </c>
+      <c r="D85" t="s">
+        <v>57</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>239</v>
+      </c>
+      <c r="B86" t="s">
+        <v>237</v>
+      </c>
+      <c r="C86" t="s">
+        <v>243</v>
+      </c>
+      <c r="D86" t="s">
+        <v>80</v>
+      </c>
+      <c r="E86" t="s">
+        <v>8</v>
+      </c>
+      <c r="F86" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>239</v>
+      </c>
+      <c r="B87" t="s">
+        <v>237</v>
+      </c>
+      <c r="C87" t="s">
+        <v>243</v>
+      </c>
+      <c r="D87" t="s">
+        <v>79</v>
+      </c>
+      <c r="E87" t="s">
+        <v>8</v>
+      </c>
+      <c r="F87" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>239</v>
+      </c>
+      <c r="B88" t="s">
+        <v>237</v>
+      </c>
+      <c r="C88" t="s">
+        <v>243</v>
+      </c>
+      <c r="D88" t="s">
+        <v>81</v>
+      </c>
+      <c r="E88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F88" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>239</v>
+      </c>
+      <c r="B89" t="s">
+        <v>237</v>
+      </c>
+      <c r="C89" t="s">
+        <v>243</v>
+      </c>
+      <c r="D89" t="s">
+        <v>89</v>
+      </c>
+      <c r="E89" t="s">
+        <v>87</v>
+      </c>
+      <c r="F89" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>239</v>
+      </c>
+      <c r="B90" t="s">
+        <v>237</v>
+      </c>
+      <c r="C90" t="s">
+        <v>243</v>
+      </c>
+      <c r="D90" t="s">
+        <v>22</v>
+      </c>
+      <c r="E90" t="s">
+        <v>8</v>
+      </c>
+      <c r="F90" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>239</v>
+      </c>
+      <c r="B91" t="s">
+        <v>237</v>
+      </c>
+      <c r="C91" t="s">
+        <v>243</v>
+      </c>
+      <c r="D91" t="s">
+        <v>29</v>
+      </c>
+      <c r="E91" t="s">
+        <v>8</v>
+      </c>
+      <c r="F91" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>239</v>
+      </c>
+      <c r="B92" t="s">
+        <v>237</v>
+      </c>
+      <c r="C92" t="s">
+        <v>243</v>
+      </c>
+      <c r="D92" t="s">
+        <v>15</v>
+      </c>
+      <c r="E92" t="s">
+        <v>8</v>
+      </c>
+      <c r="F92" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>239</v>
+      </c>
+      <c r="B93" t="s">
+        <v>237</v>
+      </c>
+      <c r="C93" t="s">
+        <v>243</v>
+      </c>
+      <c r="D93" t="s">
+        <v>50</v>
+      </c>
+      <c r="E93" t="s">
+        <v>8</v>
+      </c>
+      <c r="F93" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>239</v>
+      </c>
+      <c r="B94" t="s">
+        <v>237</v>
+      </c>
+      <c r="C94" t="s">
+        <v>243</v>
+      </c>
+      <c r="D94" t="s">
+        <v>90</v>
+      </c>
+      <c r="E94" t="s">
+        <v>87</v>
+      </c>
+      <c r="F94" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>239</v>
+      </c>
+      <c r="B95" t="s">
+        <v>237</v>
+      </c>
+      <c r="C95" t="s">
+        <v>243</v>
+      </c>
+      <c r="D95" t="s">
+        <v>7</v>
+      </c>
+      <c r="E95" t="s">
+        <v>8</v>
+      </c>
+      <c r="F95" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>239</v>
+      </c>
+      <c r="B96" t="s">
+        <v>238</v>
+      </c>
+      <c r="C96" t="s">
+        <v>243</v>
+      </c>
+      <c r="D96" t="s">
+        <v>73</v>
+      </c>
+      <c r="E96" t="s">
+        <v>87</v>
+      </c>
+      <c r="F96" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>239</v>
+      </c>
+      <c r="B97" t="s">
+        <v>238</v>
+      </c>
+      <c r="C97" t="s">
+        <v>243</v>
+      </c>
+      <c r="D97" t="s">
+        <v>75</v>
+      </c>
+      <c r="E97" t="s">
+        <v>8</v>
+      </c>
+      <c r="F97" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>239</v>
+      </c>
+      <c r="B98" t="s">
+        <v>238</v>
+      </c>
+      <c r="C98" t="s">
+        <v>243</v>
+      </c>
+      <c r="D98" t="s">
+        <v>88</v>
+      </c>
+      <c r="E98" t="s">
+        <v>87</v>
+      </c>
+      <c r="F98" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>239</v>
+      </c>
+      <c r="B99" t="s">
+        <v>238</v>
+      </c>
+      <c r="C99" t="s">
+        <v>243</v>
+      </c>
+      <c r="D99" t="s">
+        <v>57</v>
+      </c>
+      <c r="E99" t="s">
+        <v>8</v>
+      </c>
+      <c r="F99" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>239</v>
+      </c>
+      <c r="B100" t="s">
+        <v>238</v>
+      </c>
+      <c r="C100" t="s">
+        <v>243</v>
+      </c>
+      <c r="D100" t="s">
+        <v>263</v>
+      </c>
+      <c r="E100" t="s">
+        <v>8</v>
+      </c>
+      <c r="F100" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>239</v>
+      </c>
+      <c r="B101" t="s">
+        <v>238</v>
+      </c>
+      <c r="C101" t="s">
+        <v>243</v>
+      </c>
+      <c r="D101" t="s">
+        <v>79</v>
+      </c>
+      <c r="E101" t="s">
+        <v>8</v>
+      </c>
+      <c r="F101" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>239</v>
+      </c>
+      <c r="B102" t="s">
+        <v>238</v>
+      </c>
+      <c r="C102" t="s">
+        <v>243</v>
+      </c>
+      <c r="D102" t="s">
+        <v>81</v>
+      </c>
+      <c r="E102" t="s">
+        <v>8</v>
+      </c>
+      <c r="F102" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>239</v>
+      </c>
+      <c r="B103" t="s">
+        <v>238</v>
+      </c>
+      <c r="C103" t="s">
+        <v>243</v>
+      </c>
+      <c r="D103" t="s">
+        <v>89</v>
+      </c>
+      <c r="E103" t="s">
+        <v>87</v>
+      </c>
+      <c r="F103" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>239</v>
+      </c>
+      <c r="B104" t="s">
+        <v>238</v>
+      </c>
+      <c r="C104" t="s">
+        <v>243</v>
+      </c>
+      <c r="D104" t="s">
+        <v>22</v>
+      </c>
+      <c r="E104" t="s">
+        <v>8</v>
+      </c>
+      <c r="F104" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>239</v>
+      </c>
+      <c r="B105" t="s">
+        <v>238</v>
+      </c>
+      <c r="C105" t="s">
+        <v>243</v>
+      </c>
+      <c r="D105" t="s">
+        <v>29</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>239</v>
+      </c>
+      <c r="B106" t="s">
+        <v>238</v>
+      </c>
+      <c r="C106" t="s">
+        <v>243</v>
+      </c>
+      <c r="D106" t="s">
+        <v>15</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>239</v>
+      </c>
+      <c r="B107" t="s">
+        <v>238</v>
+      </c>
+      <c r="C107" t="s">
+        <v>243</v>
+      </c>
+      <c r="D107" t="s">
+        <v>50</v>
+      </c>
+      <c r="E107" t="s">
+        <v>8</v>
+      </c>
+      <c r="F107" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>239</v>
+      </c>
+      <c r="B108" t="s">
+        <v>238</v>
+      </c>
+      <c r="C108" t="s">
+        <v>243</v>
+      </c>
+      <c r="D108" t="s">
+        <v>90</v>
+      </c>
+      <c r="E108" t="s">
+        <v>87</v>
+      </c>
+      <c r="F108" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>239</v>
+      </c>
+      <c r="B109" t="s">
+        <v>238</v>
+      </c>
+      <c r="C109" t="s">
+        <v>243</v>
+      </c>
+      <c r="D109" t="s">
+        <v>7</v>
+      </c>
+      <c r="E109" t="s">
+        <v>8</v>
+      </c>
+      <c r="F109" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>114</v>
+      </c>
+      <c r="B110" t="s">
+        <v>113</v>
+      </c>
+      <c r="C110" t="s">
+        <v>243</v>
+      </c>
+      <c r="D110" t="s">
+        <v>73</v>
+      </c>
+      <c r="E110" t="s">
+        <v>87</v>
+      </c>
+      <c r="F110" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>114</v>
+      </c>
+      <c r="B111" t="s">
+        <v>113</v>
+      </c>
+      <c r="C111" t="s">
+        <v>243</v>
+      </c>
+      <c r="D111" t="s">
+        <v>75</v>
+      </c>
+      <c r="E111" t="s">
+        <v>8</v>
+      </c>
+      <c r="F111" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>114</v>
+      </c>
+      <c r="B112" t="s">
+        <v>113</v>
+      </c>
+      <c r="C112" t="s">
+        <v>243</v>
+      </c>
+      <c r="D112" t="s">
+        <v>88</v>
+      </c>
+      <c r="E112" t="s">
+        <v>87</v>
+      </c>
+      <c r="F112" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>114</v>
+      </c>
+      <c r="B113" t="s">
+        <v>113</v>
+      </c>
+      <c r="C113" t="s">
+        <v>243</v>
+      </c>
+      <c r="D113" t="s">
+        <v>57</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>114</v>
+      </c>
+      <c r="B114" t="s">
+        <v>113</v>
+      </c>
+      <c r="C114" t="s">
+        <v>243</v>
+      </c>
+      <c r="D114" t="s">
+        <v>80</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>113</v>
+      </c>
+      <c r="C115" t="s">
+        <v>243</v>
+      </c>
+      <c r="D115" t="s">
+        <v>79</v>
+      </c>
+      <c r="E115" t="s">
+        <v>8</v>
+      </c>
+      <c r="F115" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>114</v>
+      </c>
+      <c r="B116" t="s">
+        <v>113</v>
+      </c>
+      <c r="C116" t="s">
+        <v>243</v>
+      </c>
+      <c r="D116" t="s">
+        <v>81</v>
+      </c>
+      <c r="E116" t="s">
+        <v>8</v>
+      </c>
+      <c r="F116" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>114</v>
+      </c>
+      <c r="B117" t="s">
+        <v>113</v>
+      </c>
+      <c r="C117" t="s">
+        <v>243</v>
+      </c>
+      <c r="D117" t="s">
+        <v>22</v>
+      </c>
+      <c r="E117" t="s">
+        <v>8</v>
+      </c>
+      <c r="F117" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>114</v>
+      </c>
+      <c r="B118" t="s">
+        <v>113</v>
+      </c>
+      <c r="C118" t="s">
+        <v>243</v>
+      </c>
+      <c r="D118" t="s">
+        <v>64</v>
+      </c>
+      <c r="E118" t="s">
+        <v>87</v>
+      </c>
+      <c r="F118" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>114</v>
+      </c>
+      <c r="B119" t="s">
+        <v>113</v>
+      </c>
+      <c r="C119" t="s">
+        <v>243</v>
+      </c>
+      <c r="D119" t="s">
+        <v>29</v>
+      </c>
+      <c r="E119" t="s">
+        <v>8</v>
+      </c>
+      <c r="F119" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>114</v>
+      </c>
+      <c r="B120" t="s">
+        <v>113</v>
+      </c>
+      <c r="C120" t="s">
+        <v>243</v>
+      </c>
+      <c r="D120" t="s">
+        <v>15</v>
+      </c>
+      <c r="E120" t="s">
+        <v>8</v>
+      </c>
+      <c r="F120" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>114</v>
+      </c>
+      <c r="B121" t="s">
+        <v>113</v>
+      </c>
+      <c r="C121" t="s">
+        <v>243</v>
+      </c>
+      <c r="D121" t="s">
+        <v>50</v>
+      </c>
+      <c r="E121" t="s">
+        <v>8</v>
+      </c>
+      <c r="F121" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>114</v>
+      </c>
+      <c r="B122" t="s">
+        <v>113</v>
+      </c>
+      <c r="C122" t="s">
+        <v>243</v>
+      </c>
+      <c r="D122" t="s">
+        <v>90</v>
+      </c>
+      <c r="E122" t="s">
+        <v>87</v>
+      </c>
+      <c r="F122" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>114</v>
+      </c>
+      <c r="B123" t="s">
+        <v>113</v>
+      </c>
+      <c r="C123" t="s">
+        <v>243</v>
+      </c>
+      <c r="D123" t="s">
+        <v>7</v>
+      </c>
+      <c r="E123" t="s">
+        <v>8</v>
+      </c>
+      <c r="F123" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>114</v>
+      </c>
+      <c r="B124" t="s">
+        <v>237</v>
+      </c>
+      <c r="C124" t="s">
+        <v>243</v>
+      </c>
+      <c r="D124" t="s">
+        <v>73</v>
+      </c>
+      <c r="E124" t="s">
+        <v>87</v>
+      </c>
+      <c r="F124" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>114</v>
+      </c>
+      <c r="B125" t="s">
+        <v>237</v>
+      </c>
+      <c r="C125" t="s">
+        <v>243</v>
+      </c>
+      <c r="D125" t="s">
+        <v>75</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>114</v>
+      </c>
+      <c r="B126" t="s">
+        <v>237</v>
+      </c>
+      <c r="C126" t="s">
+        <v>243</v>
+      </c>
+      <c r="D126" t="s">
+        <v>88</v>
+      </c>
+      <c r="E126" t="s">
+        <v>87</v>
+      </c>
+      <c r="F126" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>114</v>
+      </c>
+      <c r="B127" t="s">
+        <v>237</v>
+      </c>
+      <c r="C127" t="s">
+        <v>243</v>
+      </c>
+      <c r="D127" t="s">
+        <v>57</v>
+      </c>
+      <c r="E127" t="s">
+        <v>8</v>
+      </c>
+      <c r="F127" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>114</v>
+      </c>
+      <c r="B128" t="s">
+        <v>237</v>
+      </c>
+      <c r="C128" t="s">
+        <v>243</v>
+      </c>
+      <c r="D128" t="s">
+        <v>80</v>
+      </c>
+      <c r="E128" t="s">
+        <v>8</v>
+      </c>
+      <c r="F128" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
+        <v>114</v>
+      </c>
+      <c r="B129" t="s">
+        <v>237</v>
+      </c>
+      <c r="C129" t="s">
+        <v>243</v>
+      </c>
+      <c r="D129" t="s">
+        <v>79</v>
+      </c>
+      <c r="E129" t="s">
+        <v>8</v>
+      </c>
+      <c r="F129" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
+        <v>114</v>
+      </c>
+      <c r="B130" t="s">
+        <v>237</v>
+      </c>
+      <c r="C130" t="s">
+        <v>243</v>
+      </c>
+      <c r="D130" t="s">
+        <v>81</v>
+      </c>
+      <c r="E130" t="s">
+        <v>8</v>
+      </c>
+      <c r="F130" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A131" t="s">
+        <v>114</v>
+      </c>
+      <c r="B131" t="s">
+        <v>237</v>
+      </c>
+      <c r="C131" t="s">
+        <v>243</v>
+      </c>
+      <c r="D131" t="s">
+        <v>22</v>
+      </c>
+      <c r="E131" t="s">
+        <v>8</v>
+      </c>
+      <c r="F131" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
+        <v>114</v>
+      </c>
+      <c r="B132" t="s">
+        <v>237</v>
+      </c>
+      <c r="C132" t="s">
+        <v>243</v>
+      </c>
+      <c r="D132" t="s">
+        <v>64</v>
+      </c>
+      <c r="E132" t="s">
+        <v>87</v>
+      </c>
+      <c r="F132" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
+        <v>114</v>
+      </c>
+      <c r="B133" t="s">
+        <v>237</v>
+      </c>
+      <c r="C133" t="s">
+        <v>243</v>
+      </c>
+      <c r="D133" t="s">
+        <v>29</v>
+      </c>
+      <c r="E133" t="s">
+        <v>8</v>
+      </c>
+      <c r="F133" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
+        <v>114</v>
+      </c>
+      <c r="B134" t="s">
+        <v>237</v>
+      </c>
+      <c r="C134" t="s">
+        <v>243</v>
+      </c>
+      <c r="D134" t="s">
+        <v>15</v>
+      </c>
+      <c r="E134" t="s">
+        <v>8</v>
+      </c>
+      <c r="F134" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A135" t="s">
+        <v>114</v>
+      </c>
+      <c r="B135" t="s">
+        <v>237</v>
+      </c>
+      <c r="C135" t="s">
+        <v>243</v>
+      </c>
+      <c r="D135" t="s">
+        <v>50</v>
+      </c>
+      <c r="E135" t="s">
+        <v>8</v>
+      </c>
+      <c r="F135" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
+        <v>114</v>
+      </c>
+      <c r="B136" t="s">
+        <v>237</v>
+      </c>
+      <c r="C136" t="s">
+        <v>243</v>
+      </c>
+      <c r="D136" t="s">
+        <v>90</v>
+      </c>
+      <c r="E136" t="s">
+        <v>87</v>
+      </c>
+      <c r="F136" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A137" t="s">
+        <v>114</v>
+      </c>
+      <c r="B137" t="s">
+        <v>237</v>
+      </c>
+      <c r="C137" t="s">
+        <v>243</v>
+      </c>
+      <c r="D137" t="s">
+        <v>7</v>
+      </c>
+      <c r="E137" t="s">
+        <v>8</v>
+      </c>
+      <c r="F137" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
+        <v>114</v>
+      </c>
+      <c r="B138" t="s">
+        <v>238</v>
+      </c>
+      <c r="C138" t="s">
+        <v>243</v>
+      </c>
+      <c r="D138" t="s">
+        <v>73</v>
+      </c>
+      <c r="E138" t="s">
+        <v>87</v>
+      </c>
+      <c r="F138" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A139" t="s">
+        <v>114</v>
+      </c>
+      <c r="B139" t="s">
+        <v>238</v>
+      </c>
+      <c r="C139" t="s">
+        <v>243</v>
+      </c>
+      <c r="D139" t="s">
+        <v>75</v>
+      </c>
+      <c r="E139" t="s">
+        <v>8</v>
+      </c>
+      <c r="F139" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
+        <v>114</v>
+      </c>
+      <c r="B140" t="s">
+        <v>238</v>
+      </c>
+      <c r="C140" t="s">
+        <v>243</v>
+      </c>
+      <c r="D140" t="s">
+        <v>88</v>
+      </c>
+      <c r="E140" t="s">
+        <v>87</v>
+      </c>
+      <c r="F140" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
+        <v>114</v>
+      </c>
+      <c r="B141" t="s">
+        <v>238</v>
+      </c>
+      <c r="C141" t="s">
+        <v>243</v>
+      </c>
+      <c r="D141" t="s">
+        <v>57</v>
+      </c>
+      <c r="E141" t="s">
+        <v>8</v>
+      </c>
+      <c r="F141" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A142" t="s">
+        <v>114</v>
+      </c>
+      <c r="B142" t="s">
+        <v>238</v>
+      </c>
+      <c r="C142" t="s">
+        <v>243</v>
+      </c>
+      <c r="D142" t="s">
+        <v>263</v>
+      </c>
+      <c r="E142" t="s">
+        <v>8</v>
+      </c>
+      <c r="F142" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
+        <v>114</v>
+      </c>
+      <c r="B143" t="s">
+        <v>238</v>
+      </c>
+      <c r="C143" t="s">
+        <v>243</v>
+      </c>
+      <c r="D143" t="s">
+        <v>79</v>
+      </c>
+      <c r="E143" t="s">
+        <v>8</v>
+      </c>
+      <c r="F143" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
+        <v>114</v>
+      </c>
+      <c r="B144" t="s">
+        <v>238</v>
+      </c>
+      <c r="C144" t="s">
+        <v>243</v>
+      </c>
+      <c r="D144" t="s">
+        <v>81</v>
+      </c>
+      <c r="E144" t="s">
+        <v>8</v>
+      </c>
+      <c r="F144" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
+        <v>114</v>
+      </c>
+      <c r="B145" t="s">
+        <v>238</v>
+      </c>
+      <c r="C145" t="s">
+        <v>243</v>
+      </c>
+      <c r="D145" t="s">
+        <v>22</v>
+      </c>
+      <c r="E145" t="s">
+        <v>8</v>
+      </c>
+      <c r="F145" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
+        <v>114</v>
+      </c>
+      <c r="B146" t="s">
+        <v>238</v>
+      </c>
+      <c r="C146" t="s">
+        <v>243</v>
+      </c>
+      <c r="D146" t="s">
+        <v>64</v>
+      </c>
+      <c r="E146" t="s">
+        <v>87</v>
+      </c>
+      <c r="F146" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A147" t="s">
+        <v>114</v>
+      </c>
+      <c r="B147" t="s">
+        <v>238</v>
+      </c>
+      <c r="C147" t="s">
+        <v>243</v>
+      </c>
+      <c r="D147" t="s">
+        <v>29</v>
+      </c>
+      <c r="E147" t="s">
+        <v>8</v>
+      </c>
+      <c r="F147" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A148" t="s">
+        <v>114</v>
+      </c>
+      <c r="B148" t="s">
+        <v>238</v>
+      </c>
+      <c r="C148" t="s">
+        <v>243</v>
+      </c>
+      <c r="D148" t="s">
+        <v>15</v>
+      </c>
+      <c r="E148" t="s">
+        <v>8</v>
+      </c>
+      <c r="F148" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A149" t="s">
+        <v>114</v>
+      </c>
+      <c r="B149" t="s">
+        <v>238</v>
+      </c>
+      <c r="C149" t="s">
+        <v>243</v>
+      </c>
+      <c r="D149" t="s">
+        <v>50</v>
+      </c>
+      <c r="E149" t="s">
+        <v>8</v>
+      </c>
+      <c r="F149" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A150" t="s">
+        <v>114</v>
+      </c>
+      <c r="B150" t="s">
+        <v>238</v>
+      </c>
+      <c r="C150" t="s">
+        <v>243</v>
+      </c>
+      <c r="D150" t="s">
+        <v>90</v>
+      </c>
+      <c r="E150" t="s">
+        <v>87</v>
+      </c>
+      <c r="F150" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
+        <v>114</v>
+      </c>
+      <c r="B151" t="s">
+        <v>238</v>
+      </c>
+      <c r="C151" t="s">
+        <v>243</v>
+      </c>
+      <c r="D151" t="s">
+        <v>7</v>
+      </c>
+      <c r="E151" t="s">
+        <v>8</v>
+      </c>
+      <c r="F151" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
+        <v>114</v>
+      </c>
+      <c r="B152" t="s">
+        <v>113</v>
+      </c>
+      <c r="C152" t="s">
+        <v>120</v>
+      </c>
+      <c r="D152" t="s">
+        <v>36</v>
+      </c>
+      <c r="E152" t="s">
+        <v>8</v>
+      </c>
+      <c r="F152" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A153" t="s">
+        <v>114</v>
+      </c>
+      <c r="B153" t="s">
+        <v>113</v>
+      </c>
+      <c r="C153" t="s">
+        <v>120</v>
+      </c>
+      <c r="D153" t="s">
+        <v>77</v>
+      </c>
+      <c r="E153" t="s">
+        <v>8</v>
+      </c>
+      <c r="F153" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A154" t="s">
+        <v>114</v>
+      </c>
+      <c r="B154" t="s">
+        <v>113</v>
+      </c>
+      <c r="C154" t="s">
+        <v>120</v>
+      </c>
+      <c r="D154" t="s">
+        <v>84</v>
+      </c>
+      <c r="E154" t="s">
+        <v>8</v>
+      </c>
+      <c r="F154" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A155" t="s">
+        <v>114</v>
+      </c>
+      <c r="B155" t="s">
+        <v>113</v>
+      </c>
+      <c r="C155" t="s">
+        <v>120</v>
+      </c>
+      <c r="D155" t="s">
+        <v>136</v>
+      </c>
+      <c r="E155" t="s">
+        <v>8</v>
+      </c>
+      <c r="F155" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A156" t="s">
+        <v>114</v>
+      </c>
+      <c r="B156" t="s">
+        <v>113</v>
+      </c>
+      <c r="C156" t="s">
+        <v>120</v>
+      </c>
+      <c r="D156" t="s">
+        <v>83</v>
+      </c>
+      <c r="E156" t="s">
+        <v>8</v>
+      </c>
+      <c r="F156" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A157" t="s">
+        <v>114</v>
+      </c>
+      <c r="B157" t="s">
+        <v>113</v>
+      </c>
+      <c r="C157" t="s">
+        <v>120</v>
+      </c>
+      <c r="D157" t="s">
+        <v>73</v>
+      </c>
+      <c r="E157" t="s">
+        <v>87</v>
+      </c>
+      <c r="F157" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A158" t="s">
+        <v>114</v>
+      </c>
+      <c r="B158" t="s">
+        <v>113</v>
+      </c>
+      <c r="C158" t="s">
+        <v>120</v>
+      </c>
+      <c r="D158" t="s">
+        <v>75</v>
+      </c>
+      <c r="E158" t="s">
+        <v>8</v>
+      </c>
+      <c r="F158" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A159" t="s">
+        <v>114</v>
+      </c>
+      <c r="B159" t="s">
+        <v>113</v>
+      </c>
+      <c r="C159" t="s">
+        <v>120</v>
+      </c>
+      <c r="D159" t="s">
+        <v>88</v>
+      </c>
+      <c r="E159" t="s">
+        <v>87</v>
+      </c>
+      <c r="F159" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A160" t="s">
+        <v>114</v>
+      </c>
+      <c r="B160" t="s">
+        <v>113</v>
+      </c>
+      <c r="C160" t="s">
+        <v>120</v>
+      </c>
+      <c r="D160" t="s">
+        <v>57</v>
+      </c>
+      <c r="E160" t="s">
+        <v>8</v>
+      </c>
+      <c r="F160" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A161" t="s">
+        <v>114</v>
+      </c>
+      <c r="B161" t="s">
+        <v>113</v>
+      </c>
+      <c r="C161" t="s">
+        <v>120</v>
+      </c>
+      <c r="D161" t="s">
+        <v>80</v>
+      </c>
+      <c r="E161" t="s">
+        <v>8</v>
+      </c>
+      <c r="F161" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A162" t="s">
+        <v>114</v>
+      </c>
+      <c r="B162" t="s">
+        <v>113</v>
+      </c>
+      <c r="C162" t="s">
+        <v>120</v>
+      </c>
+      <c r="D162" t="s">
+        <v>79</v>
+      </c>
+      <c r="E162" t="s">
+        <v>8</v>
+      </c>
+      <c r="F162" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A163" t="s">
+        <v>114</v>
+      </c>
+      <c r="B163" t="s">
+        <v>113</v>
+      </c>
+      <c r="C163" t="s">
+        <v>120</v>
+      </c>
+      <c r="D163" t="s">
+        <v>81</v>
+      </c>
+      <c r="E163" t="s">
+        <v>8</v>
+      </c>
+      <c r="F163" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A164" t="s">
+        <v>114</v>
+      </c>
+      <c r="B164" t="s">
+        <v>113</v>
+      </c>
+      <c r="C164" t="s">
+        <v>120</v>
+      </c>
+      <c r="D164" t="s">
+        <v>82</v>
+      </c>
+      <c r="E164" t="s">
+        <v>8</v>
+      </c>
+      <c r="F164" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A165" t="s">
+        <v>114</v>
+      </c>
+      <c r="B165" t="s">
+        <v>113</v>
+      </c>
+      <c r="C165" t="s">
+        <v>120</v>
+      </c>
+      <c r="D165" t="s">
+        <v>89</v>
+      </c>
+      <c r="E165" t="s">
+        <v>87</v>
+      </c>
+      <c r="F165" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A166" t="s">
+        <v>114</v>
+      </c>
+      <c r="B166" t="s">
+        <v>113</v>
+      </c>
+      <c r="C166" t="s">
+        <v>120</v>
+      </c>
+      <c r="D166" t="s">
+        <v>22</v>
+      </c>
+      <c r="E166" t="s">
+        <v>8</v>
+      </c>
+      <c r="F166" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A167" t="s">
+        <v>114</v>
+      </c>
+      <c r="B167" t="s">
+        <v>113</v>
+      </c>
+      <c r="C167" t="s">
+        <v>120</v>
+      </c>
+      <c r="D167" t="s">
+        <v>78</v>
+      </c>
+      <c r="E167" t="s">
+        <v>8</v>
+      </c>
+      <c r="F167" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A168" t="s">
+        <v>114</v>
+      </c>
+      <c r="B168" t="s">
+        <v>113</v>
+      </c>
+      <c r="C168" t="s">
+        <v>120</v>
+      </c>
+      <c r="D168" t="s">
+        <v>43</v>
+      </c>
+      <c r="E168" t="s">
+        <v>8</v>
+      </c>
+      <c r="F168" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A169" t="s">
+        <v>114</v>
+      </c>
+      <c r="B169" t="s">
+        <v>113</v>
+      </c>
+      <c r="C169" t="s">
+        <v>120</v>
+      </c>
+      <c r="D169" t="s">
+        <v>64</v>
+      </c>
+      <c r="E169" t="s">
+        <v>8</v>
+      </c>
+      <c r="F169" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A170" t="s">
+        <v>114</v>
+      </c>
+      <c r="B170" t="s">
+        <v>113</v>
+      </c>
+      <c r="C170" t="s">
+        <v>120</v>
+      </c>
+      <c r="D170" t="s">
+        <v>29</v>
+      </c>
+      <c r="E170" t="s">
+        <v>8</v>
+      </c>
+      <c r="F170" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A171" t="s">
+        <v>114</v>
+      </c>
+      <c r="B171" t="s">
+        <v>113</v>
+      </c>
+      <c r="C171" t="s">
+        <v>120</v>
+      </c>
+      <c r="D171" t="s">
+        <v>15</v>
+      </c>
+      <c r="E171" t="s">
+        <v>8</v>
+      </c>
+      <c r="F171" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A172" t="s">
+        <v>114</v>
+      </c>
+      <c r="B172" t="s">
+        <v>113</v>
+      </c>
+      <c r="C172" t="s">
+        <v>120</v>
+      </c>
+      <c r="D172" t="s">
+        <v>50</v>
+      </c>
+      <c r="E172" t="s">
+        <v>8</v>
+      </c>
+      <c r="F172" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A173" t="s">
+        <v>114</v>
+      </c>
+      <c r="B173" t="s">
+        <v>113</v>
+      </c>
+      <c r="C173" t="s">
+        <v>120</v>
+      </c>
+      <c r="D173" t="s">
+        <v>90</v>
+      </c>
+      <c r="E173" t="s">
+        <v>87</v>
+      </c>
+      <c r="F173" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A174" t="s">
+        <v>114</v>
+      </c>
+      <c r="B174" t="s">
+        <v>113</v>
+      </c>
+      <c r="C174" t="s">
+        <v>120</v>
+      </c>
+      <c r="D174" t="s">
+        <v>71</v>
+      </c>
+      <c r="E174" t="s">
+        <v>8</v>
+      </c>
+      <c r="F174" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A175" t="s">
+        <v>114</v>
+      </c>
+      <c r="B175" t="s">
+        <v>113</v>
+      </c>
+      <c r="C175" t="s">
+        <v>120</v>
+      </c>
+      <c r="D175" t="s">
+        <v>7</v>
+      </c>
+      <c r="E175" t="s">
+        <v>8</v>
+      </c>
+      <c r="F175" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A176" t="s">
+        <v>114</v>
+      </c>
+      <c r="B176" t="s">
+        <v>113</v>
+      </c>
+      <c r="C176" t="s">
+        <v>120</v>
+      </c>
+      <c r="D176" t="s">
+        <v>76</v>
+      </c>
+      <c r="E176" t="s">
+        <v>8</v>
+      </c>
+      <c r="F176" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A177" t="s">
+        <v>259</v>
+      </c>
+      <c r="B177" t="s">
+        <v>238</v>
+      </c>
+      <c r="C177" t="s">
+        <v>243</v>
+      </c>
+      <c r="D177" t="s">
+        <v>57</v>
+      </c>
+      <c r="E177" t="s">
+        <v>8</v>
+      </c>
+      <c r="F177" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A178" t="s">
+        <v>259</v>
+      </c>
+      <c r="B178" t="s">
+        <v>238</v>
+      </c>
+      <c r="C178" t="s">
+        <v>243</v>
+      </c>
+      <c r="D178" t="s">
+        <v>80</v>
+      </c>
+      <c r="E178" t="s">
+        <v>8</v>
+      </c>
+      <c r="F178" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A179" t="s">
+        <v>259</v>
+      </c>
+      <c r="B179" t="s">
+        <v>238</v>
+      </c>
+      <c r="C179" t="s">
+        <v>243</v>
+      </c>
+      <c r="D179" t="s">
+        <v>79</v>
+      </c>
+      <c r="E179" t="s">
+        <v>8</v>
+      </c>
+      <c r="F179" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A180" t="s">
+        <v>259</v>
+      </c>
+      <c r="B180" t="s">
+        <v>238</v>
+      </c>
+      <c r="C180" t="s">
+        <v>243</v>
+      </c>
+      <c r="D180" t="s">
+        <v>22</v>
+      </c>
+      <c r="E180" t="s">
+        <v>8</v>
+      </c>
+      <c r="F180" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A181" t="s">
+        <v>259</v>
+      </c>
+      <c r="B181" t="s">
+        <v>238</v>
+      </c>
+      <c r="C181" t="s">
+        <v>243</v>
+      </c>
+      <c r="D181" t="s">
+        <v>29</v>
+      </c>
+      <c r="E181" t="s">
+        <v>8</v>
+      </c>
+      <c r="F181" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A182" t="s">
+        <v>259</v>
+      </c>
+      <c r="B182" t="s">
+        <v>238</v>
+      </c>
+      <c r="C182" t="s">
+        <v>243</v>
+      </c>
+      <c r="D182" t="s">
+        <v>15</v>
+      </c>
+      <c r="E182" t="s">
+        <v>8</v>
+      </c>
+      <c r="F182" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A183" t="s">
+        <v>259</v>
+      </c>
+      <c r="B183" t="s">
+        <v>238</v>
+      </c>
+      <c r="C183" t="s">
+        <v>243</v>
+      </c>
+      <c r="D183" t="s">
+        <v>50</v>
+      </c>
+      <c r="E183" t="s">
+        <v>8</v>
+      </c>
+      <c r="F183" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A184" t="s">
+        <v>259</v>
+      </c>
+      <c r="B184" t="s">
+        <v>238</v>
+      </c>
+      <c r="C184" t="s">
+        <v>243</v>
+      </c>
+      <c r="D184" t="s">
+        <v>7</v>
+      </c>
+      <c r="E184" t="s">
+        <v>8</v>
+      </c>
+      <c r="F184" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A185" t="s">
+        <v>259</v>
+      </c>
+      <c r="B185" t="s">
+        <v>245</v>
+      </c>
+      <c r="C185" t="s">
+        <v>243</v>
+      </c>
+      <c r="D185" t="s">
+        <v>57</v>
+      </c>
+      <c r="E185" t="s">
+        <v>8</v>
+      </c>
+      <c r="F185" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A186" t="s">
+        <v>259</v>
+      </c>
+      <c r="B186" t="s">
+        <v>245</v>
+      </c>
+      <c r="C186" t="s">
+        <v>243</v>
+      </c>
+      <c r="D186" t="s">
+        <v>80</v>
+      </c>
+      <c r="E186" t="s">
+        <v>8</v>
+      </c>
+      <c r="F186" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A187" t="s">
+        <v>259</v>
+      </c>
+      <c r="B187" t="s">
+        <v>245</v>
+      </c>
+      <c r="C187" t="s">
+        <v>243</v>
+      </c>
+      <c r="D187" t="s">
+        <v>79</v>
+      </c>
+      <c r="E187" t="s">
+        <v>8</v>
+      </c>
+      <c r="F187" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A188" t="s">
+        <v>259</v>
+      </c>
+      <c r="B188" t="s">
+        <v>245</v>
+      </c>
+      <c r="C188" t="s">
+        <v>243</v>
+      </c>
+      <c r="D188" t="s">
+        <v>22</v>
+      </c>
+      <c r="E188" t="s">
+        <v>8</v>
+      </c>
+      <c r="F188" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A189" t="s">
+        <v>259</v>
+      </c>
+      <c r="B189" t="s">
+        <v>245</v>
+      </c>
+      <c r="C189" t="s">
+        <v>243</v>
+      </c>
+      <c r="D189" t="s">
+        <v>29</v>
+      </c>
+      <c r="E189" t="s">
+        <v>8</v>
+      </c>
+      <c r="F189" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A190" t="s">
+        <v>259</v>
+      </c>
+      <c r="B190" t="s">
+        <v>245</v>
+      </c>
+      <c r="C190" t="s">
+        <v>243</v>
+      </c>
+      <c r="D190" t="s">
+        <v>15</v>
+      </c>
+      <c r="E190" t="s">
+        <v>8</v>
+      </c>
+      <c r="F190" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A191" t="s">
+        <v>259</v>
+      </c>
+      <c r="B191" t="s">
+        <v>245</v>
+      </c>
+      <c r="C191" t="s">
+        <v>243</v>
+      </c>
+      <c r="D191" t="s">
+        <v>50</v>
+      </c>
+      <c r="E191" t="s">
+        <v>8</v>
+      </c>
+      <c r="F191" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A192" t="s">
+        <v>259</v>
+      </c>
+      <c r="B192" t="s">
+        <v>245</v>
+      </c>
+      <c r="C192" t="s">
+        <v>243</v>
+      </c>
+      <c r="D192" t="s">
+        <v>7</v>
+      </c>
+      <c r="E192" t="s">
+        <v>8</v>
+      </c>
+      <c r="F192" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A193" t="s">
+        <v>259</v>
+      </c>
+      <c r="B193" t="s">
+        <v>231</v>
+      </c>
+      <c r="C193" t="s">
+        <v>232</v>
+      </c>
+      <c r="D193" t="s">
+        <v>73</v>
+      </c>
+      <c r="E193" t="s">
+        <v>232</v>
+      </c>
+      <c r="F193" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
+        <v>259</v>
+      </c>
+      <c r="B194" t="s">
+        <v>231</v>
+      </c>
+      <c r="C194" t="s">
+        <v>121</v>
+      </c>
+      <c r="D194" t="s">
+        <v>73</v>
+      </c>
+      <c r="E194" t="s">
+        <v>8</v>
+      </c>
+      <c r="F194" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
+        <v>259</v>
+      </c>
+      <c r="B195" t="s">
+        <v>247</v>
+      </c>
+      <c r="C195" t="s">
+        <v>121</v>
+      </c>
+      <c r="D195" t="s">
+        <v>73</v>
+      </c>
+      <c r="E195" t="s">
+        <v>8</v>
+      </c>
+      <c r="F195" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
+        <v>259</v>
+      </c>
+      <c r="B196" t="s">
+        <v>248</v>
+      </c>
+      <c r="C196" t="s">
+        <v>121</v>
+      </c>
+      <c r="D196" t="s">
+        <v>73</v>
+      </c>
+      <c r="E196" t="s">
+        <v>8</v>
+      </c>
+      <c r="F196" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
+        <v>259</v>
+      </c>
+      <c r="B197" t="s">
+        <v>249</v>
+      </c>
+      <c r="C197" t="s">
+        <v>121</v>
+      </c>
+      <c r="D197" t="s">
+        <v>73</v>
+      </c>
+      <c r="E197" t="s">
+        <v>8</v>
+      </c>
+      <c r="F197" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
+        <v>259</v>
+      </c>
+      <c r="B198" t="s">
+        <v>250</v>
+      </c>
+      <c r="C198" t="s">
+        <v>121</v>
+      </c>
+      <c r="D198" t="s">
+        <v>73</v>
+      </c>
+      <c r="E198" t="s">
+        <v>8</v>
+      </c>
+      <c r="F198" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
+        <v>259</v>
+      </c>
+      <c r="B199" t="s">
+        <v>251</v>
+      </c>
+      <c r="C199" t="s">
+        <v>121</v>
+      </c>
+      <c r="D199" t="s">
+        <v>73</v>
+      </c>
+      <c r="E199" t="s">
+        <v>8</v>
+      </c>
+      <c r="F199" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A200" t="s">
+        <v>259</v>
+      </c>
+      <c r="B200" t="s">
+        <v>252</v>
+      </c>
+      <c r="C200" t="s">
+        <v>121</v>
+      </c>
+      <c r="D200" t="s">
+        <v>73</v>
+      </c>
+      <c r="E200" t="s">
+        <v>8</v>
+      </c>
+      <c r="F200" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A201" t="s">
+        <v>259</v>
+      </c>
+      <c r="B201" t="s">
+        <v>253</v>
+      </c>
+      <c r="C201" t="s">
+        <v>121</v>
+      </c>
+      <c r="D201" t="s">
+        <v>73</v>
+      </c>
+      <c r="E201" t="s">
+        <v>8</v>
+      </c>
+      <c r="F201" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A202" t="s">
+        <v>259</v>
+      </c>
+      <c r="B202" t="s">
+        <v>254</v>
+      </c>
+      <c r="C202" t="s">
+        <v>121</v>
+      </c>
+      <c r="D202" t="s">
+        <v>73</v>
+      </c>
+      <c r="E202" t="s">
+        <v>8</v>
+      </c>
+      <c r="F202" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
+        <v>259</v>
+      </c>
+      <c r="B203" t="s">
+        <v>255</v>
+      </c>
+      <c r="C203" t="s">
+        <v>121</v>
+      </c>
+      <c r="D203" t="s">
+        <v>73</v>
+      </c>
+      <c r="E203" t="s">
+        <v>8</v>
+      </c>
+      <c r="F203" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A204" t="s">
+        <v>259</v>
+      </c>
+      <c r="B204" t="s">
+        <v>256</v>
+      </c>
+      <c r="C204" t="s">
+        <v>121</v>
+      </c>
+      <c r="D204" t="s">
+        <v>73</v>
+      </c>
+      <c r="E204" t="s">
+        <v>8</v>
+      </c>
+      <c r="F204" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A205" t="s">
+        <v>259</v>
+      </c>
+      <c r="B205" t="s">
+        <v>257</v>
+      </c>
+      <c r="C205" t="s">
+        <v>121</v>
+      </c>
+      <c r="D205" t="s">
+        <v>73</v>
+      </c>
+      <c r="E205" t="s">
+        <v>8</v>
+      </c>
+      <c r="F205" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A206" t="s">
+        <v>259</v>
+      </c>
+      <c r="B206" t="s">
+        <v>258</v>
+      </c>
+      <c r="C206" t="s">
+        <v>121</v>
+      </c>
+      <c r="D206" t="s">
+        <v>73</v>
+      </c>
+      <c r="E206" t="s">
+        <v>8</v>
+      </c>
+      <c r="F206" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A207" t="s">
+        <v>259</v>
+      </c>
+      <c r="B207" t="s">
+        <v>238</v>
+      </c>
+      <c r="C207" t="s">
+        <v>262</v>
+      </c>
+      <c r="D207" t="s">
+        <v>29</v>
+      </c>
+      <c r="E207" t="s">
+        <v>8</v>
+      </c>
+      <c r="F207" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A208" t="s">
+        <v>259</v>
+      </c>
+      <c r="B208" t="s">
+        <v>238</v>
+      </c>
+      <c r="C208" t="s">
+        <v>262</v>
+      </c>
+      <c r="D208" t="s">
+        <v>57</v>
+      </c>
+      <c r="E208" t="s">
+        <v>8</v>
+      </c>
+      <c r="F208" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A209" t="s">
+        <v>259</v>
+      </c>
+      <c r="B209" t="s">
+        <v>238</v>
+      </c>
+      <c r="C209" t="s">
+        <v>262</v>
+      </c>
+      <c r="D209" t="s">
+        <v>22</v>
+      </c>
+      <c r="E209" t="s">
+        <v>8</v>
+      </c>
+      <c r="F209" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A210" t="s">
+        <v>259</v>
+      </c>
+      <c r="B210" t="s">
+        <v>238</v>
+      </c>
+      <c r="C210" t="s">
+        <v>262</v>
+      </c>
+      <c r="D210" t="s">
+        <v>263</v>
+      </c>
+      <c r="E210" t="s">
+        <v>8</v>
+      </c>
+      <c r="F210" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A211" t="s">
+        <v>259</v>
+      </c>
+      <c r="B211" t="s">
+        <v>264</v>
+      </c>
+      <c r="C211" t="s">
+        <v>262</v>
+      </c>
+      <c r="D211" t="s">
+        <v>261</v>
+      </c>
+      <c r="E211" t="s">
+        <v>8</v>
+      </c>
+      <c r="F211" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A212" t="s">
+        <v>259</v>
+      </c>
+      <c r="B212" t="s">
+        <v>264</v>
+      </c>
+      <c r="C212" t="s">
+        <v>262</v>
+      </c>
+      <c r="D212" t="s">
+        <v>57</v>
+      </c>
+      <c r="E212" t="s">
+        <v>8</v>
+      </c>
+      <c r="F212" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A213" t="s">
+        <v>259</v>
+      </c>
+      <c r="B213" t="s">
+        <v>264</v>
+      </c>
+      <c r="C213" t="s">
+        <v>262</v>
+      </c>
+      <c r="D213" t="s">
+        <v>22</v>
+      </c>
+      <c r="E213" t="s">
+        <v>8</v>
+      </c>
+      <c r="F213" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A214" t="s">
+        <v>246</v>
+      </c>
+      <c r="B214" t="s">
+        <v>260</v>
+      </c>
+      <c r="C214" t="s">
+        <v>248</v>
+      </c>
+      <c r="D214" t="s">
+        <v>261</v>
+      </c>
+      <c r="E214" t="s">
+        <v>8</v>
+      </c>
+      <c r="F214" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A215" t="s">
+        <v>246</v>
+      </c>
+      <c r="B215" t="s">
+        <v>260</v>
+      </c>
+      <c r="C215" t="s">
+        <v>248</v>
+      </c>
+      <c r="D215" t="s">
+        <v>7</v>
+      </c>
+      <c r="E215" t="s">
+        <v>8</v>
+      </c>
+      <c r="F215" s="3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{30459df5-1e53-4d8b-a162-0ad2348546f1}" enabled="0" method="" siteId="{30459df5-1e53-4d8b-a162-0ad2348546f1}" removed="1"/>

</xml_diff>